<commit_message>
Count only human tumor tissue as patient material (correction #20)
</commit_message>
<xml_diff>
--- a/workbooks/SupplementaryTable1_entities.xlsx
+++ b/workbooks/SupplementaryTable1_entities.xlsx
@@ -607,10 +607,10 @@
         <v>23</v>
       </c>
       <c r="L2" s="4" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="M2" s="4" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="N2" s="4" t="n">
         <v>2</v>
@@ -1146,19 +1146,19 @@
         </is>
       </c>
       <c r="I10" s="4" t="n">
-        <v>310</v>
+        <v>290</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>180</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="L10" s="4" t="n">
         <v>17</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>4</v>
@@ -1167,7 +1167,7 @@
         <v>21</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>4.769</v>
+        <v>4.462</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1757,10 +1757,10 @@
         <v>557</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>172</v>
+        <v>104</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>596</v>
+        <v>510</v>
       </c>
       <c r="N19" s="4" t="n">
         <v>50</v>
@@ -1893,10 +1893,10 @@
         <v>14</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="N21" s="4" t="n">
         <v>5</v>
@@ -2016,28 +2016,28 @@
         </is>
       </c>
       <c r="I23" s="4" t="n">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="J23" s="4" t="n">
         <v>668</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L23" s="4" t="n">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>155</v>
+        <v>81</v>
       </c>
       <c r="N23" s="4" t="n">
         <v>13</v>
       </c>
       <c r="O23" s="4" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P23" s="4" t="n">
-        <v>8.300000000000001</v>
+        <v>8.291</v>
       </c>
       <c r="Q23" s="3" t="inlineStr">
         <is>
@@ -2091,10 +2091,10 @@
         <v>102</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>211</v>
+        <v>151</v>
       </c>
       <c r="N24" s="4" t="n">
         <v>11</v>
@@ -2157,10 +2157,10 @@
         <v>67</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="N25" s="4" t="n">
         <v>8</v>
@@ -2705,10 +2705,10 @@
         <v>281</v>
       </c>
       <c r="L33" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N33" s="4" t="n">
         <v>14</v>
@@ -2766,28 +2766,28 @@
         </is>
       </c>
       <c r="I34" s="4" t="n">
-        <v>1577</v>
+        <v>1545</v>
       </c>
       <c r="J34" s="4" t="n">
         <v>966</v>
       </c>
       <c r="K34" s="4" t="n">
-        <v>520</v>
+        <v>488</v>
       </c>
       <c r="L34" s="4" t="n">
         <v>109</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>383</v>
+        <v>351</v>
       </c>
       <c r="N34" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O34" s="4" t="n">
         <v>67</v>
       </c>
       <c r="P34" s="4" t="n">
-        <v>16.6</v>
+        <v>16.263</v>
       </c>
       <c r="Q34" s="3" t="inlineStr">
         <is>
@@ -2844,7 +2844,7 @@
         <v>4</v>
       </c>
       <c r="M35" s="4" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="N35" s="4" t="n">
         <v>2</v>
@@ -3186,28 +3186,28 @@
         </is>
       </c>
       <c r="I40" s="4" t="n">
-        <v>4379</v>
+        <v>4372</v>
       </c>
       <c r="J40" s="4" t="n">
-        <v>2984</v>
+        <v>2983</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>493</v>
+        <v>487</v>
       </c>
       <c r="L40" s="4" t="n">
-        <v>271</v>
+        <v>164</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>548</v>
+        <v>319</v>
       </c>
       <c r="N40" s="4" t="n">
         <v>32</v>
       </c>
       <c r="O40" s="4" t="n">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="P40" s="4" t="n">
-        <v>4.131</v>
+        <v>4.125</v>
       </c>
       <c r="Q40" s="3" t="inlineStr">
         <is>
@@ -3533,10 +3533,10 @@
         <v>16</v>
       </c>
       <c r="L45" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="N45" s="4" t="n">
         <v>3</v>

</xml_diff>